<commit_message>
Revert "Update 23.295 Stable"
This reverts commit bf80fa6d40131e742e6f687edcb9d3f498cf9cec.
</commit_message>
<xml_diff>
--- a/PTBR-COM-PORTRAIT/Lang/PTBR/Dialog/Drama/_chara.xlsx
+++ b/PTBR-COM-PORTRAIT/Lang/PTBR/Dialog/Drama/_chara.xlsx
@@ -757,7 +757,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>$hired</t>
+          <t>$contratado</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>$hired</t>
+          <t>$contratada</t>
         </is>
       </c>
     </row>

</xml_diff>